<commit_message>
updated doi in metadata
</commit_message>
<xml_diff>
--- a/data/excel/metadata.xlsx
+++ b/data/excel/metadata.xlsx
@@ -860,7 +860,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -19292,7 +19291,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>3vz2</t>
+          <t>3zv2</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -19347,7 +19346,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>3vz2</t>
+          <t>3zv2</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -19402,7 +19401,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>3vz2</t>
+          <t>3zv2</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -28952,7 +28951,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>3vz2</t>
+          <t>3zv2</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">

</xml_diff>